<commit_message>
Rebuild the results page around the study path; fix dropdown arrow
- Headline by score: 160+ hears "You're doing great work" with their
  LSAC percentile (2023-2026 table); below 160 starts with building the
  reasoning foundation (BYU, 7Sage, LSAT Lab, Blueprint, LawHub lessons)
- Path steps as expandable cards: practice questions (LawHub Advantage
  $124/yr, fee waiver, LSAT Demon, 7Sage, LSAT Lab, Leland, full courses),
  wrong answer journal, correcting your reasoning (explanations, AI with
  Gemini/Claude logos and the in-page tutor, coaching with Caleb), and a
  consistent schedule with calendar links
- Journal templates use research-backed fields
- Plans add a full timed practice test every week or two; below 160 the
  first weeks focus on fundamentals
- Custom select chevron sits 16px from the right edge

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqEReuR2iVt7VfNpqWbcrn
</commit_message>
<xml_diff>
--- a/public/templates/lsat-wrong-answer-journal.xlsx
+++ b/public/templates/lsat-wrong-answer-journal.xlsx
@@ -458,14 +458,14 @@
   <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -476,7 +476,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Test and question</t>
+          <t>The question (test, section, number)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -486,27 +486,27 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>My answer</t>
+          <t>My answer, and why I picked it</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Right answer</t>
+          <t>Right answer, and why it's right</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Why I missed it</t>
+          <t>What went wrong</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>What to look for next time</t>
+          <t>How I'll get it right next time</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Reviewed again?</t>
+          <t>Redid it? (date, right or wrong)</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PT 141, LR 1, Q14</t>
+          <t>PT 141, LR section 1, question 14</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -528,17 +528,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B. It sounded like the argument's conclusion, so it felt safe.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>D. It names the mistake: the argument treats a correlation as a cause.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>I picked an answer that described the argument instead of its mistake.</t>
+          <t>Fell for a trap. I picked an answer that described the argument instead of its flaw.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Oct 19, right</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1576,19 +1576,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. Write why you picked your answer and why the right one is right. Ask AI if you are not sure.</t>
+          <t>2. Be honest about why your answer was tempting. That is the habit you are training out.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. Review the journal once a week. Look for the mistakes that keep coming back, and drill those question types.</t>
+          <t>3. Write one rule for next time. Ask AI to explain the question if you are not sure why the right answer is right.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Redo each question a week later without looking at your notes. Review the journal every week and drill the question types that keep showing up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Row 2 on the Journal sheet is an example. Replace it with your own first entry.</t>
         </is>

</xml_diff>